<commit_message>
Updated documentation for v1.0.1
</commit_message>
<xml_diff>
--- a/Documents/RT24 Radio Configuration Table.xlsx
+++ b/Documents/RT24 Radio Configuration Table.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_GitWorkspace\Retevis-RT24\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C572DD9-2130-4DE7-AB79-80D31253C0A6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BCEC0F-4FE3-4FDC-942F-F0A7FD205847}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17620" xr2:uid="{2F353EC1-3109-4D44-9297-7AF6286BFB6D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17620" activeTab="1" xr2:uid="{2F353EC1-3109-4D44-9297-7AF6286BFB6D}"/>
   </bookViews>
   <sheets>
     <sheet name="v1.0.0" sheetId="2" r:id="rId1"/>
+    <sheet name="v1.0.1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="17">
   <si>
     <t>Low</t>
   </si>
@@ -78,6 +79,12 @@
   </si>
   <si>
     <t>D026N</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -128,7 +135,46 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="26">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -182,20 +228,40 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{49ED3242-2059-4734-9D47-0EC8FCAF91C6}" name="Configuration" displayName="Configuration" ref="B2:L18" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{49ED3242-2059-4734-9D47-0EC8FCAF91C6}" name="Configuration" displayName="Configuration" ref="B2:L18" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="B2:L18" xr:uid="{B245F137-5EC2-4E57-8782-5C10811BD82B}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{57CEFAAE-FAB3-438D-B218-13C6304D48DF}" name="Channel" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{E75A94DA-E7F4-4A4E-B644-843DA077E4B7}" name="RX Freq(MHz)" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{2E965840-6482-434A-8160-0570A1A0EE4D}" name="CTC/DCS DEC" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{F8650204-590C-4364-A843-24B7F1625346}" name="TX Freq(MHz)" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{F06AFEF2-6F4B-448F-9B93-3CD88D65FE37}" name="CTC/DCS FNC" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{19E99242-6000-4713-B628-B1D2513B7892}" name="Scan Add" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{72D3449E-300C-4AF8-88F8-ED4B7F7C5C25}" name="Wide/Narrow Band" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{769263EB-0E94-4B22-8471-9A126404C721}" name="TX Power" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{600761C3-6A4D-49D4-99C9-3745C946415A}" name="Busy Lock" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{3C3F4981-1E5B-4A48-9080-18F5C2AD0723}" name="Scramble" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{19094088-E4AB-40F3-A217-EBD8A88A64A9}" name="Compander" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{57CEFAAE-FAB3-438D-B218-13C6304D48DF}" name="Channel" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{E75A94DA-E7F4-4A4E-B644-843DA077E4B7}" name="RX Freq(MHz)" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{2E965840-6482-434A-8160-0570A1A0EE4D}" name="CTC/DCS DEC" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{F8650204-590C-4364-A843-24B7F1625346}" name="TX Freq(MHz)" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{F06AFEF2-6F4B-448F-9B93-3CD88D65FE37}" name="CTC/DCS FNC" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{19E99242-6000-4713-B628-B1D2513B7892}" name="Scan Add" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{72D3449E-300C-4AF8-88F8-ED4B7F7C5C25}" name="Wide/Narrow Band" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{769263EB-0E94-4B22-8471-9A126404C721}" name="TX Power" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{600761C3-6A4D-49D4-99C9-3745C946415A}" name="Busy Lock" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{3C3F4981-1E5B-4A48-9080-18F5C2AD0723}" name="Scramble" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{19094088-E4AB-40F3-A217-EBD8A88A64A9}" name="Compander" dataDxfId="13"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EA48404C-444A-4B58-A04C-8EEB37E9DF99}" name="Configuration3" displayName="Configuration3" ref="B2:L18" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="B2:L18" xr:uid="{A822D809-D117-4AF2-8976-029546AD5F37}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{3050FD47-7F17-4EE7-8876-3663EB8BC15C}" name="Channel" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{7D55591E-345F-4D4E-9908-5C8EB9093C27}" name="RX Freq(MHz)" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{C29E83ED-5191-4D4A-9D6C-27E713CA8DCA}" name="CTC/DCS DEC" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{F4C6EBFE-2ECA-4F79-B1B3-7CCE9EDBA2AC}" name="TX Freq(MHz)" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{B4FBD649-4E13-4561-925E-166F44FE7CC3}" name="CTC/DCS FNC" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{51CF05AF-F1C0-47A7-A870-A55006438803}" name="Scan Add" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{4216DE60-1747-47E4-A375-1F6E060E9A81}" name="Wide/Narrow Band" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{0F94BC2C-1290-4AAB-909F-7F759A21DA90}" name="TX Power" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{E2FE4162-8841-4846-881F-B6FFA1723C4C}" name="Busy Lock" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{82BD6E26-AFBB-4160-8093-D7D6B0796BCA}" name="Scramble" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{62409295-702D-4A2D-A59E-2CF19CCC8203}" name="Compander" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1122,4 +1188,625 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9333E3A-3E9C-455A-9FD2-4EF7AAD2A856}">
+  <dimension ref="B2:L18"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.9140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.9140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.58203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.4140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>446.00625000000002</v>
+      </c>
+      <c r="D3" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E3" s="1">
+        <v>446.00625000000002</v>
+      </c>
+      <c r="F3" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>446.01875000000001</v>
+      </c>
+      <c r="D4" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E4" s="1">
+        <v>446.01875000000001</v>
+      </c>
+      <c r="F4" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>446.03125</v>
+      </c>
+      <c r="D5" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E5" s="1">
+        <v>446.03125</v>
+      </c>
+      <c r="F5" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B6" s="1">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1">
+        <v>446.04374999999999</v>
+      </c>
+      <c r="D6" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E6" s="1">
+        <v>446.04374999999999</v>
+      </c>
+      <c r="F6" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B7" s="1">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
+        <v>446.05624999999998</v>
+      </c>
+      <c r="D7" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E7" s="1">
+        <v>446.05624999999998</v>
+      </c>
+      <c r="F7" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B8" s="1">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1">
+        <v>446.06875000000002</v>
+      </c>
+      <c r="D8" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E8" s="1">
+        <v>446.06875000000002</v>
+      </c>
+      <c r="F8" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B9" s="1">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1">
+        <v>446.08125000000001</v>
+      </c>
+      <c r="D9" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E9" s="1">
+        <v>446.08125000000001</v>
+      </c>
+      <c r="F9" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="1">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1">
+        <v>446.09375</v>
+      </c>
+      <c r="D10" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E10" s="1">
+        <v>446.09375</v>
+      </c>
+      <c r="F10" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B11" s="1">
+        <v>9</v>
+      </c>
+      <c r="C11" s="1">
+        <v>446.10624999999999</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="1">
+        <v>446.10624999999999</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B12" s="1">
+        <v>10</v>
+      </c>
+      <c r="C12" s="1">
+        <v>446.11874999999998</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="1">
+        <v>446.11874999999998</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B13" s="1">
+        <v>11</v>
+      </c>
+      <c r="C13" s="1">
+        <v>446.13125000000002</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="1">
+        <v>446.13125000000002</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B14" s="1">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1">
+        <v>446.14375000000001</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="1">
+        <v>446.14375000000001</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B15" s="1">
+        <v>13</v>
+      </c>
+      <c r="C15" s="1">
+        <v>446.15625</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="1">
+        <v>446.15625</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B16" s="1">
+        <v>14</v>
+      </c>
+      <c r="C16" s="1">
+        <v>446.16874999999999</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="1">
+        <v>446.16874999999999</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B17" s="1">
+        <v>15</v>
+      </c>
+      <c r="C17" s="1">
+        <v>446.18124999999998</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="1">
+        <v>446.18124999999998</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B18" s="1">
+        <v>16</v>
+      </c>
+      <c r="C18" s="1">
+        <v>446.19375000000002</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="1">
+        <v>446.19375000000002</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>